<commit_message>
Přidat datové pruhy do sešitu cvičení kapitoly 5
Ruční úprava autora v Excelu: podmíněné formátování datovými pruhy
ve sloupci N listů U3_tipovani (N4:N14), U4_test_20 (N4:N24)
a U5_aproximace (N4:N34). Hodnoty, vzorce a listy beze změny.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/presentations/kapitola_05_pravdepodobnost_cviceni.xlsx
+++ b/presentations/kapitola_05_pravdepodobnost_cviceni.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4C866EA0-E2E2-43EA-BF1E-117D32BD090E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD129F23-F2D0-425C-86A7-140409B7FAFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-109" yWindow="-109" windowWidth="34995" windowHeight="19060" xr2:uid="{62758DF3-0AA8-4524-8049-0D8AB62D465E}"/>
   </bookViews>
@@ -8683,8 +8683,64 @@
     <mergeCell ref="A36:A37"/>
     <mergeCell ref="A42:A44"/>
   </mergeCells>
+  <conditionalFormatting sqref="N4:N14">
+    <cfRule type="dataBar" priority="2">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF63C384"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{13B51F72-DEB9-48A2-AD29-4384F12D4423}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O4:O14">
+    <cfRule type="dataBar" priority="1">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF638EC6"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{3B842BD7-17A7-4B0F-A7E5-05D5C8087C22}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
+      <x14:conditionalFormattings>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{13B51F72-DEB9-48A2-AD29-4384F12D4423}">
+            <x14:dataBar minLength="0" maxLength="100" gradient="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>N4:N14</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{3B842BD7-17A7-4B0F-A7E5-05D5C8087C22}">
+            <x14:dataBar minLength="0" maxLength="100" gradient="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>O4:O14</xm:sqref>
+        </x14:conditionalFormatting>
+      </x14:conditionalFormattings>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
 
@@ -9514,8 +9570,39 @@
     <mergeCell ref="A17:A21"/>
     <mergeCell ref="A23:A24"/>
   </mergeCells>
+  <conditionalFormatting sqref="N4:N24">
+    <cfRule type="dataBar" priority="1">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF63C384"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{7967EC80-6898-4519-95A4-FF0767744A91}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
+      <x14:conditionalFormattings>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{7967EC80-6898-4519-95A4-FF0767744A91}">
+            <x14:dataBar minLength="0" maxLength="100" gradient="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>N4:N24</xm:sqref>
+        </x14:conditionalFormatting>
+      </x14:conditionalFormattings>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
 
@@ -10586,7 +10673,38 @@
     <mergeCell ref="A35:A36"/>
     <mergeCell ref="A41:A42"/>
   </mergeCells>
+  <conditionalFormatting sqref="N4:N34">
+    <cfRule type="dataBar" priority="1">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF63C384"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{39B395FB-CDA0-46F2-84F2-F60399557E00}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
+      <x14:conditionalFormattings>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{39B395FB-CDA0-46F2-84F2-F60399557E00}">
+            <x14:dataBar minLength="0" maxLength="100" gradient="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>N4:N34</xm:sqref>
+        </x14:conditionalFormatting>
+      </x14:conditionalFormattings>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
</xml_diff>